<commit_message>
made the final changes
</commit_message>
<xml_diff>
--- a/docs/samples/imports/employee-import-batch-1.xlsx
+++ b/docs/samples/imports/employee-import-batch-1.xlsx
@@ -424,7 +424,7 @@
         <v>Anika Kapoor</v>
       </c>
       <c r="B2" t="str">
-        <v>import.batch1.01@oddo-import.test</v>
+        <v>import.batch1.01@odoo-import.test</v>
       </c>
       <c r="C2" t="str">
         <v>Engineering</v>
@@ -444,7 +444,7 @@
         <v>Rohan Desai</v>
       </c>
       <c r="B3" t="str">
-        <v>import.batch1.02@oddo-import.test</v>
+        <v>import.batch1.02@odoo-import.test</v>
       </c>
       <c r="C3" t="str">
         <v>Human Resources</v>
@@ -464,7 +464,7 @@
         <v>Meera Iyer</v>
       </c>
       <c r="B4" t="str">
-        <v>import.batch1.03@oddo-import.test</v>
+        <v>import.batch1.03@odoo-import.test</v>
       </c>
       <c r="C4" t="str">
         <v>Sales</v>
@@ -484,7 +484,7 @@
         <v>Kabir Nair</v>
       </c>
       <c r="B5" t="str">
-        <v>import.batch1.04@oddo-import.test</v>
+        <v>import.batch1.04@odoo-import.test</v>
       </c>
       <c r="C5" t="str">
         <v>Finance</v>
@@ -504,7 +504,7 @@
         <v>Sana Qureshi</v>
       </c>
       <c r="B6" t="str">
-        <v>import.batch1.05@oddo-import.test</v>
+        <v>import.batch1.05@odoo-import.test</v>
       </c>
       <c r="C6" t="str">
         <v>Marketing</v>
@@ -524,7 +524,7 @@
         <v>Dev Patel</v>
       </c>
       <c r="B7" t="str">
-        <v>import.batch1.06@oddo-import.test</v>
+        <v>import.batch1.06@odoo-import.test</v>
       </c>
       <c r="C7" t="str">
         <v>Operations</v>
@@ -544,7 +544,7 @@
         <v>Isha Reddy</v>
       </c>
       <c r="B8" t="str">
-        <v>import.batch1.07@oddo-import.test</v>
+        <v>import.batch1.07@odoo-import.test</v>
       </c>
       <c r="C8" t="str">
         <v>Customer Success</v>
@@ -564,7 +564,7 @@
         <v>Arjun Singh</v>
       </c>
       <c r="B9" t="str">
-        <v>import.batch1.08@oddo-import.test</v>
+        <v>import.batch1.08@odoo-import.test</v>
       </c>
       <c r="C9" t="str">
         <v>Product</v>
@@ -584,7 +584,7 @@
         <v>Nisha Joshi</v>
       </c>
       <c r="B10" t="str">
-        <v>import.batch1.09@oddo-import.test</v>
+        <v>import.batch1.09@odoo-import.test</v>
       </c>
       <c r="C10" t="str">
         <v>Legal</v>
@@ -604,7 +604,7 @@
         <v>Vihaan Gupta</v>
       </c>
       <c r="B11" t="str">
-        <v>import.batch1.10@oddo-import.test</v>
+        <v>import.batch1.10@odoo-import.test</v>
       </c>
       <c r="C11" t="str">
         <v>IT Support</v>

</xml_diff>